<commit_message>
feat: enterprise-standard project structure with BRD, SDD, and dashboard screenshot
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-15</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: high-end AX portfolio final release with massive Geoje data and AI panel
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,17 +458,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>선체1팀</t>
+          <t>도장설비팀</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>도장A팀</t>
+          <t>시운전팀</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-02-22</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>의장2팀</t>
+          <t>엔진기술팀</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>품질관리</t>
+          <t>도장설비팀</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -546,17 +546,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>안전보건</t>
+          <t>선체조립1팀</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>선체1팀</t>
+          <t>도장설비팀</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-02-22</t>
         </is>
       </c>
     </row>
@@ -590,17 +590,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>도장A팀</t>
+          <t>도장설비팀</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
@@ -612,17 +612,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>의장2팀</t>
+          <t>선체조립1팀</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>품질관리</t>
+          <t>특수선설계팀</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -656,17 +656,237 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>안전보건</t>
+          <t>엔진기술팀</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>이수</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>박상면</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>특수선설계팀</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>이수</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>한소희</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>시운전팀</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>이수</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>이상혁</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>의장지원팀</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>미이수</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>김연경</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>의장지원팀</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>이수</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>손흥민</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>선체조립1팀</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>이수</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>봉준호</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>의장지원팀</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>이수</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>송강호</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>엔진기술팀</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>미이수</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>배수지</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>엔진기술팀</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>이수</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>남주혁</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>엔진기술팀</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>이수</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
         <is>
           <t>2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>아이유</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>시운전팀</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>이수</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
style: optimize dashboard spacing and labels, fix: update docs with DB & BI plans
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>도장설비팀</t>
+          <t>엔진기술팀</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>시운전팀</t>
+          <t>엔진기술팀</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-26</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>엔진기술팀</t>
+          <t>의장지원팀</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-02-22</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>도장설비팀</t>
+          <t>선체조립1팀</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -546,17 +546,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>선체조립1팀</t>
+          <t>의장지원팀</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-26</t>
         </is>
       </c>
     </row>
@@ -568,17 +568,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>도장설비팀</t>
+          <t>선체조립1팀</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-02</t>
         </is>
       </c>
     </row>
@@ -612,17 +612,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>선체조립1팀</t>
+          <t>의장지원팀</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-21</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>특수선설계팀</t>
+          <t>도장설비팀</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>엔진기술팀</t>
+          <t>특수선설계팀</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>특수선설계팀</t>
+          <t>시운전팀</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>시운전팀</t>
+          <t>선체조립1팀</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -722,17 +722,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>의장지원팀</t>
+          <t>선체조립1팀</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-03-01</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>의장지원팀</t>
+          <t>도장설비팀</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>선체조립1팀</t>
+          <t>의장지원팀</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>의장지원팀</t>
+          <t>시운전팀</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
@@ -810,17 +810,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>엔진기술팀</t>
+          <t>특수선설계팀</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>엔진기술팀</t>
+          <t>의장지원팀</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -854,17 +854,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>엔진기술팀</t>
+          <t>도장설비팀</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -876,17 +876,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>시운전팀</t>
+          <t>엔진기술팀</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: modular enterprise AX architecture v2.5 with bilingual UI and strategy docs
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="safety_training_master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,17 +458,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>엔진기술팀</t>
+          <t>한화오션 공정관리팀</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>엔진기술팀</t>
+          <t>한화오션 공정관리팀</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>의장지원팀</t>
+          <t>한화오션 공정관리팀</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>선체조립1팀</t>
+          <t>한화오션 공정관리팀</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>의장지원팀</t>
+          <t>한화오션 공정관리팀</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>선체조립1팀</t>
+          <t>한화오션 공정관리팀</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -578,41 +578,41 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>강현우</t>
+          <t>배수지</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>도장설비팀</t>
+          <t>한화오션 공정관리팀</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>윤미래</t>
+          <t>남주혁</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>의장지원팀</t>
+          <t>한화오션 공정관리팀</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -622,271 +622,51 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>조세호</t>
+          <t>아이유</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>도장설비팀</t>
+          <t>한화오션 공정관리팀</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>임지연</t>
+          <t>손흥민</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>특수선설계팀</t>
+          <t>한화오션 공정관리팀</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>박상면</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>시운전팀</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-03-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>한소희</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>선체조립1팀</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-03-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>이상혁</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>선체조립1팀</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>김연경</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>도장설비팀</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>손흥민</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>의장지원팀</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>봉준호</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>시운전팀</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>송강호</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>특수선설계팀</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>배수지</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>의장지원팀</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>2026-02-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>남주혁</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>도장설비팀</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>미이수</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>아이유</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>엔진기술팀</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>미이수</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: master spacing fix v2.5.3
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: absolute spacing fix v2.5.4
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-23</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-15</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-15</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: perfection release v2.5.5
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-08</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-08</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: master alignment fix v2.5.6
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-01</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: balanced spacing v2.6
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-02-26</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: balance refinement v2.6.1
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: precision balance v2.6.2
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-01</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -617,12 +617,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-02</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-02-26</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: master balance v2.6.3
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-26</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-15</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-02</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-15</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: horizontal bar refactor v2.7
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: horizontal precision tuning v2.8
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-23</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: master center alignment v2.9
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: perfect center alignment v2.9.1
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-26</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
@@ -617,12 +617,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: rebranding to '한화오션' and responsive overhaul v3.0
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -617,12 +617,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: precision rebranding and high-visibility scaling v3.0
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-02-26</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-03</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: v3.1 spatial precision and deep center alignment
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-03</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-08</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: v3.2 golden ratio centering and vertical rhythm optimization
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
@@ -617,12 +617,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: v4.0 enterprise pro rebranding with noto sans kr
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-08</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
@@ -617,12 +617,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: fix font weight syntax for v4.0 enterprise pro
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>
@@ -617,12 +617,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: v4.0.2 final precision spacing alignment
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-02</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-15</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-03</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-03</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: v4.1 Hangeul Pure Identity and Label formatting
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-03</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-02-26</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: branding refinement v4.3.1 - official logo and layout optimization
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
@@ -507,12 +507,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-01</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
@@ -617,12 +617,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-08</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: finalize v4.4.1 grid layout and header branding
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-23</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
style: finalize centered UI/UX v4.5.0 and remove logo
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(rpa): Modernize dashboard with Tailwind CSS and Korean localization
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,22 +417,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>이름</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>팀</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>이수여부</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>교육일자</t>
         </is>
@@ -463,12 +451,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
@@ -490,7 +478,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
@@ -507,12 +495,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -534,7 +522,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -551,12 +539,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>미이수</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -578,7 +566,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>
@@ -600,7 +588,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -617,12 +605,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>이수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-08</t>
         </is>
       </c>
     </row>
@@ -644,7 +632,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>
@@ -666,7 +654,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final Refactoring v25.0.0: Unified Dashboard/API access points, added one-click startup script, and restored Governance guidelines. Optimized README for CEO visualization.
</commit_message>
<xml_diff>
--- a/data/safety_training_master.xlsx
+++ b/data/safety_training_master.xlsx
@@ -413,248 +413,168 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>이름</t>
+          <t>협력사명</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>팀</t>
+          <t>직원명</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>이수여부</t>
+          <t>직무</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>교육일자</t>
+          <t>안전교육만료일</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>연락처</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>한화테크</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>김철수</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>한화오션 공정관리팀</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>용접</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>test1@example.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>오션마린</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>이영희</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>한화오션 공정관리팀</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>이수</t>
+          <t>도장</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>test2@example.com</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>그린공업</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>박지민</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>한화오션 공정관리팀</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>배관</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>test3@example.com</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>최동석</t>
+          <t>블루조선</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>한화오션 공정관리팀</t>
+          <t>최두식</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>설계</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>test4@example.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>정수아</t>
+          <t>화이트물류</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>한화오션 공정관리팀</t>
+          <t>한소룡</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>미이수</t>
+          <t>검사</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>홍길동</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>한화오션 공정관리팀</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>배수지</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>한화오션 공정관리팀</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>미이수</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>남주혁</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>한화오션 공정관리팀</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>아이유</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>한화오션 공정관리팀</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>손흥민</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>한화오션 공정관리팀</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>이수</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>test5@example.com</t>
         </is>
       </c>
     </row>

</xml_diff>